<commit_message>
Update CBR lending + escrow statistics
</commit_message>
<xml_diff>
--- a/raw/cbr/vfs/02_04_New_loans_ind.xlsx
+++ b/raw/cbr/vfs/02_04_New_loans_ind.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ЭтаКнига" defaultThemeVersion="153222"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\CIOR\Statistika\Otdel_ORKBD\DOC_MAO\316\Сайт_робот\01.07.2026\Mortgage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\CIOR\Statistika\Otdel_ORKBD\DOC_MAO\316\Сайт_робот\01.08.2026\BankSector\Mortgage\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7845"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11820" windowHeight="8760"/>
   </bookViews>
   <sheets>
     <sheet name="в рублях" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="190">
   <si>
     <t>Январь 2019</t>
   </si>
@@ -291,6 +291,9 @@
   </si>
   <si>
     <t>Июнь 2026</t>
+  </si>
+  <si>
+    <t>Июль 2026</t>
   </si>
   <si>
     <t>РОССИЙСКАЯ ФЕДЕРАЦИЯ</t>
@@ -1012,18 +1015,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Лист1"/>
-  <dimension ref="A1:CM99"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:CN99"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.85546875" customWidth="1"/>
-    <col min="2" max="91" width="16.7109375" customWidth="1"/>
+    <col min="2" max="92" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:91" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:91" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:92" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:92" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1039,7 +1041,7 @@
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
     </row>
-    <row r="3" spans="1:91" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:92" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>0</v>
@@ -1311,10 +1313,13 @@
       <c r="CM3" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="CN3" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="5">
         <v>897835</v>
@@ -1586,10 +1591,13 @@
       <c r="CM4" s="5">
         <v>2362908</v>
       </c>
+      <c r="CN4" s="5">
+        <v>2278547</v>
+      </c>
     </row>
-    <row r="5" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="7">
         <v>292158</v>
@@ -1861,10 +1869,13 @@
       <c r="CM5" s="7">
         <v>740505</v>
       </c>
+      <c r="CN5" s="7">
+        <v>711268</v>
+      </c>
     </row>
-    <row r="6" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" s="9">
         <v>7770</v>
@@ -2136,10 +2147,13 @@
       <c r="CM6" s="9">
         <v>20553</v>
       </c>
+      <c r="CN6" s="9">
+        <v>19350</v>
+      </c>
     </row>
-    <row r="7" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B7" s="10">
         <v>5104</v>
@@ -2411,10 +2425,13 @@
       <c r="CM7" s="10">
         <v>13724</v>
       </c>
+      <c r="CN7" s="10">
+        <v>13631</v>
+      </c>
     </row>
-    <row r="8" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B8" s="9">
         <v>6195</v>
@@ -2686,10 +2703,13 @@
       <c r="CM8" s="9">
         <v>17299</v>
       </c>
+      <c r="CN8" s="9">
+        <v>16889</v>
+      </c>
     </row>
-    <row r="9" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B9" s="10">
         <v>11664</v>
@@ -2961,10 +2981,13 @@
       <c r="CM9" s="10">
         <v>31613</v>
       </c>
+      <c r="CN9" s="10">
+        <v>29377</v>
+      </c>
     </row>
-    <row r="10" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" s="9">
         <v>4152</v>
@@ -3236,10 +3259,13 @@
       <c r="CM10" s="9">
         <v>11403</v>
       </c>
+      <c r="CN10" s="9">
+        <v>10843</v>
+      </c>
     </row>
-    <row r="11" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B11" s="10">
         <v>6330</v>
@@ -3511,10 +3537,13 @@
       <c r="CM11" s="10">
         <v>16134</v>
       </c>
+      <c r="CN11" s="10">
+        <v>15609</v>
+      </c>
     </row>
-    <row r="12" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B12" s="9">
         <v>2780</v>
@@ -3786,10 +3815,13 @@
       <c r="CM12" s="9">
         <v>7878</v>
       </c>
+      <c r="CN12" s="9">
+        <v>7056</v>
+      </c>
     </row>
-    <row r="13" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B13" s="10">
         <v>5463</v>
@@ -4061,10 +4093,13 @@
       <c r="CM13" s="10">
         <v>13763</v>
       </c>
+      <c r="CN13" s="10">
+        <v>13299</v>
+      </c>
     </row>
-    <row r="14" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14" s="9">
         <v>5957</v>
@@ -4336,10 +4371,13 @@
       <c r="CM14" s="9">
         <v>14588</v>
       </c>
+      <c r="CN14" s="9">
+        <v>13939</v>
+      </c>
     </row>
-    <row r="15" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B15" s="10">
         <v>70090</v>
@@ -4611,10 +4649,13 @@
       <c r="CM15" s="10">
         <v>188122</v>
       </c>
+      <c r="CN15" s="10">
+        <v>178745</v>
+      </c>
     </row>
-    <row r="16" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="9">
         <v>3846</v>
@@ -4886,10 +4927,13 @@
       <c r="CM16" s="9">
         <v>9110</v>
       </c>
+      <c r="CN16" s="9">
+        <v>8987</v>
+      </c>
     </row>
-    <row r="17" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" s="10">
         <v>5624</v>
@@ -5161,10 +5205,13 @@
       <c r="CM17" s="10">
         <v>15344</v>
       </c>
+      <c r="CN17" s="10">
+        <v>14531</v>
+      </c>
     </row>
-    <row r="18" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B18" s="9">
         <v>4667</v>
@@ -5436,10 +5483,13 @@
       <c r="CM18" s="9">
         <v>11674</v>
       </c>
+      <c r="CN18" s="9">
+        <v>11679</v>
+      </c>
     </row>
-    <row r="19" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B19" s="10">
         <v>4636</v>
@@ -5711,10 +5761,13 @@
       <c r="CM19" s="10">
         <v>10808</v>
       </c>
+      <c r="CN19" s="10">
+        <v>10399</v>
+      </c>
     </row>
-    <row r="20" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B20" s="9">
         <v>6899</v>
@@ -5986,10 +6039,13 @@
       <c r="CM20" s="9">
         <v>16784</v>
       </c>
+      <c r="CN20" s="9">
+        <v>16569</v>
+      </c>
     </row>
-    <row r="21" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" s="10">
         <v>8404</v>
@@ -6261,10 +6317,13 @@
       <c r="CM21" s="10">
         <v>21068</v>
       </c>
+      <c r="CN21" s="10">
+        <v>20132</v>
+      </c>
     </row>
-    <row r="22" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B22" s="9">
         <v>6152</v>
@@ -6536,10 +6595,13 @@
       <c r="CM22" s="9">
         <v>17038</v>
       </c>
+      <c r="CN22" s="9">
+        <v>16140</v>
+      </c>
     </row>
-    <row r="23" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B23" s="10">
         <v>126426</v>
@@ -6811,10 +6873,13 @@
       <c r="CM23" s="10">
         <v>303602</v>
       </c>
+      <c r="CN23" s="10">
+        <v>294093</v>
+      </c>
     </row>
-    <row r="24" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B24" s="11">
         <v>111955</v>
@@ -7086,10 +7151,13 @@
       <c r="CM24" s="11">
         <v>269449</v>
       </c>
+      <c r="CN24" s="11">
+        <v>258591</v>
+      </c>
     </row>
-    <row r="25" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B25" s="10">
         <v>4098</v>
@@ -7361,10 +7429,13 @@
       <c r="CM25" s="10">
         <v>9323</v>
       </c>
+      <c r="CN25" s="10">
+        <v>9029</v>
+      </c>
     </row>
-    <row r="26" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B26" s="9">
         <v>6269</v>
@@ -7636,10 +7707,13 @@
       <c r="CM26" s="9">
         <v>12862</v>
       </c>
+      <c r="CN26" s="9">
+        <v>12604</v>
+      </c>
     </row>
-    <row r="27" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B27" s="10">
         <v>7904</v>
@@ -7911,10 +7985,13 @@
       <c r="CM27" s="10">
         <v>18182</v>
       </c>
+      <c r="CN27" s="10">
+        <v>18236</v>
+      </c>
     </row>
-    <row r="28" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B28" s="9">
         <v>360</v>
@@ -8186,10 +8263,13 @@
       <c r="CM28" s="9">
         <v>768</v>
       </c>
+      <c r="CN28" s="9">
+        <v>891</v>
+      </c>
     </row>
-    <row r="29" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B29" s="10">
         <v>7544</v>
@@ -8461,10 +8541,13 @@
       <c r="CM29" s="10">
         <v>17415</v>
       </c>
+      <c r="CN29" s="10">
+        <v>17345</v>
+      </c>
     </row>
-    <row r="30" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B30" s="9">
         <v>6485</v>
@@ -8736,10 +8819,13 @@
       <c r="CM30" s="9">
         <v>16910</v>
       </c>
+      <c r="CN30" s="9">
+        <v>15903</v>
+      </c>
     </row>
-    <row r="31" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B31" s="10">
         <v>6718</v>
@@ -9011,10 +9097,13 @@
       <c r="CM31" s="10">
         <v>18883</v>
       </c>
+      <c r="CN31" s="10">
+        <v>18577</v>
+      </c>
     </row>
-    <row r="32" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B32" s="9">
         <v>13496</v>
@@ -9286,10 +9375,13 @@
       <c r="CM32" s="9">
         <v>36653</v>
       </c>
+      <c r="CN32" s="9">
+        <v>35106</v>
+      </c>
     </row>
-    <row r="33" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B33" s="10">
         <v>6786</v>
@@ -9561,10 +9653,13 @@
       <c r="CM33" s="10">
         <v>14246</v>
       </c>
+      <c r="CN33" s="10">
+        <v>14112</v>
+      </c>
     </row>
-    <row r="34" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B34" s="9">
         <v>3074</v>
@@ -9836,10 +9931,13 @@
       <c r="CM34" s="9">
         <v>7939</v>
       </c>
+      <c r="CN34" s="9">
+        <v>7489</v>
+      </c>
     </row>
-    <row r="35" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" s="10">
         <v>2981</v>
@@ -10111,10 +10209,13 @@
       <c r="CM35" s="10">
         <v>7657</v>
       </c>
+      <c r="CN35" s="10">
+        <v>7443</v>
+      </c>
     </row>
-    <row r="36" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B36" s="9">
         <v>54145</v>
@@ -10386,10 +10487,13 @@
       <c r="CM36" s="9">
         <v>126792</v>
       </c>
+      <c r="CN36" s="9">
+        <v>120092</v>
+      </c>
     </row>
-    <row r="37" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B37" s="7">
         <v>73795</v>
@@ -10661,10 +10765,13 @@
       <c r="CM37" s="7">
         <v>231571</v>
       </c>
+      <c r="CN37" s="7">
+        <v>221718</v>
+      </c>
     </row>
-    <row r="38" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B38" s="9">
         <v>1930</v>
@@ -10936,10 +11043,13 @@
       <c r="CM38" s="9">
         <v>5921</v>
       </c>
+      <c r="CN38" s="9">
+        <v>6037</v>
+      </c>
     </row>
-    <row r="39" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B39" s="10">
         <v>1585</v>
@@ -11211,10 +11321,13 @@
       <c r="CM39" s="10">
         <v>5397</v>
       </c>
+      <c r="CN39" s="10">
+        <v>5225</v>
+      </c>
     </row>
-    <row r="40" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B40" s="9">
         <v>1598</v>
@@ -11486,10 +11599,13 @@
       <c r="CM40" s="9">
         <v>19537</v>
       </c>
+      <c r="CN40" s="9">
+        <v>17010</v>
+      </c>
     </row>
-    <row r="41" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B41" s="10">
         <v>30764</v>
@@ -11761,10 +11877,13 @@
       <c r="CM41" s="10">
         <v>92003</v>
       </c>
+      <c r="CN41" s="10">
+        <v>88449</v>
+      </c>
     </row>
-    <row r="42" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B42" s="9">
         <v>5005</v>
@@ -12036,10 +12155,13 @@
       <c r="CM42" s="9">
         <v>13437</v>
       </c>
+      <c r="CN42" s="9">
+        <v>13013</v>
+      </c>
     </row>
-    <row r="43" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B43" s="10">
         <v>11912</v>
@@ -12311,10 +12433,13 @@
       <c r="CM43" s="10">
         <v>29608</v>
       </c>
+      <c r="CN43" s="10">
+        <v>28683</v>
+      </c>
     </row>
-    <row r="44" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B44" s="9">
         <v>20487</v>
@@ -12586,10 +12711,13 @@
       <c r="CM44" s="9">
         <v>59887</v>
       </c>
+      <c r="CN44" s="9">
+        <v>57773</v>
+      </c>
     </row>
-    <row r="45" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B45" s="10">
         <v>514</v>
@@ -12861,10 +12989,13 @@
       <c r="CM45" s="10">
         <v>5781</v>
       </c>
+      <c r="CN45" s="10">
+        <v>5520</v>
+      </c>
     </row>
-    <row r="46" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B46" s="11">
         <v>22858</v>
@@ -13136,10 +13267,13 @@
       <c r="CM46" s="11">
         <v>65652</v>
       </c>
+      <c r="CN46" s="11">
+        <v>64103</v>
+      </c>
     </row>
-    <row r="47" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B47" s="10">
         <v>3026</v>
@@ -13411,10 +13545,13 @@
       <c r="CM47" s="10">
         <v>11152</v>
       </c>
+      <c r="CN47" s="10">
+        <v>10793</v>
+      </c>
     </row>
-    <row r="48" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B48" s="9">
         <v>317</v>
@@ -13686,10 +13823,13 @@
       <c r="CM48" s="9">
         <v>1068</v>
       </c>
+      <c r="CN48" s="9">
+        <v>1111</v>
+      </c>
     </row>
-    <row r="49" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B49" s="10">
         <v>2001</v>
@@ -13961,10 +14101,13 @@
       <c r="CM49" s="10">
         <v>5718</v>
       </c>
+      <c r="CN49" s="10">
+        <v>5825</v>
+      </c>
     </row>
-    <row r="50" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B50" s="9">
         <v>1368</v>
@@ -14236,10 +14379,13 @@
       <c r="CM50" s="9">
         <v>3923</v>
       </c>
+      <c r="CN50" s="9">
+        <v>3939</v>
+      </c>
     </row>
-    <row r="51" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B51" s="10">
         <v>2386</v>
@@ -14511,10 +14657,13 @@
       <c r="CM51" s="10">
         <v>6378</v>
       </c>
+      <c r="CN51" s="10">
+        <v>6371</v>
+      </c>
     </row>
-    <row r="52" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B52" s="9">
         <v>1217</v>
@@ -14786,10 +14935,13 @@
       <c r="CM52" s="9">
         <v>4523</v>
       </c>
+      <c r="CN52" s="9">
+        <v>4664</v>
+      </c>
     </row>
-    <row r="53" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B53" s="10">
         <v>12543</v>
@@ -15061,10 +15213,13 @@
       <c r="CM53" s="10">
         <v>32890</v>
       </c>
+      <c r="CN53" s="10">
+        <v>31402</v>
+      </c>
     </row>
-    <row r="54" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B54" s="11">
         <v>157596</v>
@@ -15336,10 +15491,13 @@
       <c r="CM54" s="11">
         <v>433793</v>
       </c>
+      <c r="CN54" s="11">
+        <v>416040</v>
+      </c>
     </row>
-    <row r="55" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B55" s="10">
         <v>22869</v>
@@ -15611,10 +15769,13 @@
       <c r="CM55" s="10">
         <v>62849</v>
       </c>
+      <c r="CN55" s="10">
+        <v>58894</v>
+      </c>
     </row>
-    <row r="56" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B56" s="9">
         <v>3119</v>
@@ -15886,10 +16047,13 @@
       <c r="CM56" s="9">
         <v>8998</v>
       </c>
+      <c r="CN56" s="9">
+        <v>8234</v>
+      </c>
     </row>
-    <row r="57" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B57" s="10">
         <v>3236</v>
@@ -16161,10 +16325,13 @@
       <c r="CM57" s="10">
         <v>8893</v>
       </c>
+      <c r="CN57" s="10">
+        <v>8660</v>
+      </c>
     </row>
-    <row r="58" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B58" s="9">
         <v>23240</v>
@@ -16436,10 +16603,13 @@
       <c r="CM58" s="9">
         <v>67429</v>
       </c>
+      <c r="CN58" s="9">
+        <v>64240</v>
+      </c>
     </row>
-    <row r="59" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B59" s="10">
         <v>8597</v>
@@ -16711,10 +16881,13 @@
       <c r="CM59" s="10">
         <v>25619</v>
       </c>
+      <c r="CN59" s="10">
+        <v>23973</v>
+      </c>
     </row>
-    <row r="60" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B60" s="9">
         <v>6284</v>
@@ -16986,10 +17159,13 @@
       <c r="CM60" s="9">
         <v>17731</v>
       </c>
+      <c r="CN60" s="9">
+        <v>17012</v>
+      </c>
     </row>
-    <row r="61" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B61" s="10">
         <v>16305</v>
@@ -17261,10 +17437,13 @@
       <c r="CM61" s="10">
         <v>43927</v>
       </c>
+      <c r="CN61" s="10">
+        <v>41349</v>
+      </c>
     </row>
-    <row r="62" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B62" s="9">
         <v>6202</v>
@@ -17536,10 +17715,13 @@
       <c r="CM62" s="9">
         <v>17349</v>
       </c>
+      <c r="CN62" s="9">
+        <v>16324</v>
+      </c>
     </row>
-    <row r="63" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B63" s="10">
         <v>16516</v>
@@ -17811,10 +17993,13 @@
       <c r="CM63" s="10">
         <v>47522</v>
       </c>
+      <c r="CN63" s="10">
+        <v>45953</v>
+      </c>
     </row>
-    <row r="64" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B64" s="9">
         <v>10591</v>
@@ -18086,10 +18271,13 @@
       <c r="CM64" s="9">
         <v>28042</v>
       </c>
+      <c r="CN64" s="9">
+        <v>27661</v>
+      </c>
     </row>
-    <row r="65" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B65" s="10">
         <v>5920</v>
@@ -18361,10 +18549,13 @@
       <c r="CM65" s="10">
         <v>15367</v>
       </c>
+      <c r="CN65" s="10">
+        <v>14660</v>
+      </c>
     </row>
-    <row r="66" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" s="9">
         <v>18064</v>
@@ -18636,10 +18827,13 @@
       <c r="CM66" s="9">
         <v>45975</v>
       </c>
+      <c r="CN66" s="9">
+        <v>45757</v>
+      </c>
     </row>
-    <row r="67" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B67" s="10">
         <v>10804</v>
@@ -18911,10 +19105,13 @@
       <c r="CM67" s="10">
         <v>29387</v>
       </c>
+      <c r="CN67" s="10">
+        <v>28583</v>
+      </c>
     </row>
-    <row r="68" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B68" s="9">
         <v>5849</v>
@@ -19186,10 +19383,13 @@
       <c r="CM68" s="9">
         <v>14705</v>
       </c>
+      <c r="CN68" s="9">
+        <v>14740</v>
+      </c>
     </row>
-    <row r="69" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B69" s="7">
         <v>88642</v>
@@ -19461,10 +19661,13 @@
       <c r="CM69" s="7">
         <v>226369</v>
       </c>
+      <c r="CN69" s="7">
+        <v>217760</v>
+      </c>
     </row>
-    <row r="70" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="9">
         <v>4080</v>
@@ -19736,10 +19939,13 @@
       <c r="CM70" s="9">
         <v>10747</v>
       </c>
+      <c r="CN70" s="9">
+        <v>10599</v>
+      </c>
     </row>
-    <row r="71" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B71" s="10">
         <v>28786</v>
@@ -20011,10 +20217,13 @@
       <c r="CM71" s="10">
         <v>75048</v>
       </c>
+      <c r="CN71" s="10">
+        <v>72133</v>
+      </c>
     </row>
-    <row r="72" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B72" s="9">
         <v>36574</v>
@@ -20286,10 +20495,13 @@
       <c r="CM72" s="9">
         <v>87097</v>
       </c>
+      <c r="CN72" s="9">
+        <v>83773</v>
+      </c>
     </row>
-    <row r="73" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B73" s="10">
         <v>16940</v>
@@ -20561,10 +20773,13 @@
       <c r="CM73" s="10">
         <v>36358</v>
       </c>
+      <c r="CN73" s="10">
+        <v>35659</v>
+      </c>
     </row>
-    <row r="74" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B74" s="9">
         <v>5985</v>
@@ -20836,10 +21051,13 @@
       <c r="CM74" s="9">
         <v>14219</v>
       </c>
+      <c r="CN74" s="9">
+        <v>14277</v>
+      </c>
     </row>
-    <row r="75" spans="1:91" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:92" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B75" s="10">
         <v>13649</v>
@@ -21111,10 +21329,13 @@
       <c r="CM75" s="10">
         <v>36520</v>
       </c>
+      <c r="CN75" s="10">
+        <v>33836</v>
+      </c>
     </row>
-    <row r="76" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B76" s="9">
         <v>19202</v>
@@ -21386,10 +21607,13 @@
       <c r="CM76" s="9">
         <v>53477</v>
       </c>
+      <c r="CN76" s="9">
+        <v>51255</v>
+      </c>
     </row>
-    <row r="77" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B77" s="7">
         <v>98265</v>
@@ -21661,10 +21885,13 @@
       <c r="CM77" s="7">
         <v>260702</v>
       </c>
+      <c r="CN77" s="7">
+        <v>253394</v>
+      </c>
     </row>
-    <row r="78" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B78" s="9">
         <v>921</v>
@@ -21936,10 +22163,13 @@
       <c r="CM78" s="9">
         <v>3307</v>
       </c>
+      <c r="CN78" s="9">
+        <v>3326</v>
+      </c>
     </row>
-    <row r="79" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B79" s="10">
         <v>1461</v>
@@ -22211,10 +22441,13 @@
       <c r="CM79" s="10">
         <v>5398</v>
       </c>
+      <c r="CN79" s="10">
+        <v>5375</v>
+      </c>
     </row>
-    <row r="80" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B80" s="9">
         <v>2550</v>
@@ -22486,10 +22719,13 @@
       <c r="CM80" s="9">
         <v>7938</v>
       </c>
+      <c r="CN80" s="9">
+        <v>7919</v>
+      </c>
     </row>
-    <row r="81" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B81" s="10">
         <v>10654</v>
@@ -22761,10 +22997,13 @@
       <c r="CM81" s="10">
         <v>27857</v>
       </c>
+      <c r="CN81" s="10">
+        <v>26958</v>
+      </c>
     </row>
-    <row r="82" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B82" s="9">
         <v>17842</v>
@@ -23036,10 +23275,13 @@
       <c r="CM82" s="9">
         <v>47576</v>
       </c>
+      <c r="CN82" s="9">
+        <v>46530</v>
+      </c>
     </row>
-    <row r="83" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B83" s="10">
         <v>14673</v>
@@ -23311,10 +23553,13 @@
       <c r="CM83" s="10">
         <v>38299</v>
       </c>
+      <c r="CN83" s="10">
+        <v>37134</v>
+      </c>
     </row>
-    <row r="84" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B84" s="9">
         <v>14358</v>
@@ -23586,10 +23831,13 @@
       <c r="CM84" s="9">
         <v>35533</v>
       </c>
+      <c r="CN84" s="9">
+        <v>34781</v>
+      </c>
     </row>
-    <row r="85" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B85" s="10">
         <v>19026</v>
@@ -23861,10 +24109,13 @@
       <c r="CM85" s="10">
         <v>49226</v>
       </c>
+      <c r="CN85" s="10">
+        <v>47362</v>
+      </c>
     </row>
-    <row r="86" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B86" s="9">
         <v>10626</v>
@@ -24136,10 +24387,13 @@
       <c r="CM86" s="9">
         <v>28914</v>
       </c>
+      <c r="CN86" s="9">
+        <v>28238</v>
+      </c>
     </row>
-    <row r="87" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B87" s="10">
         <v>6153</v>
@@ -24411,10 +24665,13 @@
       <c r="CM87" s="10">
         <v>16654</v>
       </c>
+      <c r="CN87" s="10">
+        <v>15770</v>
+      </c>
     </row>
-    <row r="88" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B88" s="11">
         <v>52566</v>
@@ -24686,10 +24943,13 @@
       <c r="CM88" s="11">
         <v>134868</v>
       </c>
+      <c r="CN88" s="11">
+        <v>135674</v>
+      </c>
     </row>
-    <row r="89" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B89" s="10">
         <v>4596</v>
@@ -24961,10 +25221,13 @@
       <c r="CM89" s="10">
         <v>15069</v>
       </c>
+      <c r="CN89" s="10">
+        <v>15556</v>
+      </c>
     </row>
-    <row r="90" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B90" s="9">
         <v>7303</v>
@@ -25236,10 +25499,13 @@
       <c r="CM90" s="9">
         <v>18316</v>
       </c>
+      <c r="CN90" s="9">
+        <v>19224</v>
+      </c>
     </row>
-    <row r="91" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B91" s="10">
         <v>5157</v>
@@ -25511,10 +25777,13 @@
       <c r="CM91" s="10">
         <v>15336</v>
       </c>
+      <c r="CN91" s="10">
+        <v>14731</v>
+      </c>
     </row>
-    <row r="92" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B92" s="9">
         <v>2749</v>
@@ -25786,10 +26055,13 @@
       <c r="CM92" s="9">
         <v>6357</v>
       </c>
+      <c r="CN92" s="9">
+        <v>6437</v>
+      </c>
     </row>
-    <row r="93" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B93" s="10">
         <v>12103</v>
@@ -26061,10 +26333,13 @@
       <c r="CM93" s="10">
         <v>30155</v>
       </c>
+      <c r="CN93" s="10">
+        <v>30023</v>
+      </c>
     </row>
-    <row r="94" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B94" s="9">
         <v>9024</v>
@@ -26336,10 +26611,13 @@
       <c r="CM94" s="9">
         <v>21390</v>
       </c>
+      <c r="CN94" s="9">
+        <v>21570</v>
+      </c>
     </row>
-    <row r="95" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B95" s="10">
         <v>4665</v>
@@ -26611,10 +26889,13 @@
       <c r="CM95" s="10">
         <v>12033</v>
       </c>
+      <c r="CN95" s="10">
+        <v>11930</v>
+      </c>
     </row>
-    <row r="96" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B96" s="9">
         <v>1538</v>
@@ -26886,10 +27167,13 @@
       <c r="CM96" s="9">
         <v>3253</v>
       </c>
+      <c r="CN96" s="9">
+        <v>3316</v>
+      </c>
     </row>
-    <row r="97" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B97" s="10">
         <v>4152</v>
@@ -27161,10 +27445,13 @@
       <c r="CM97" s="10">
         <v>9704</v>
       </c>
+      <c r="CN97" s="10">
+        <v>9534</v>
+      </c>
     </row>
-    <row r="98" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B98" s="9">
         <v>826</v>
@@ -27436,10 +27723,13 @@
       <c r="CM98" s="9">
         <v>1949</v>
       </c>
+      <c r="CN98" s="9">
+        <v>2004</v>
+      </c>
     </row>
-    <row r="99" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B99" s="10">
         <v>454</v>
@@ -27710,6 +28000,9 @@
       </c>
       <c r="CM99" s="10">
         <v>1308</v>
+      </c>
+      <c r="CN99" s="10">
+        <v>1349</v>
       </c>
     </row>
   </sheetData>
@@ -27724,18 +28017,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Лист2"/>
-  <dimension ref="A1:CM99"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:CN99"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.85546875" customWidth="1"/>
-    <col min="2" max="91" width="16.7109375" customWidth="1"/>
+    <col min="2" max="92" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:91" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:91" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:92" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:92" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -27751,7 +28043,7 @@
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
     </row>
-    <row r="3" spans="1:91" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:92" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>0</v>
@@ -28023,10 +28315,13 @@
       <c r="CM3" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="CN3" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="5">
         <v>3990</v>
@@ -28298,10 +28593,13 @@
       <c r="CM4" s="5">
         <v>70</v>
       </c>
+      <c r="CN4" s="5">
+        <v>30</v>
+      </c>
     </row>
-    <row r="5" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="7">
         <v>2753</v>
@@ -28573,10 +28871,13 @@
       <c r="CM5" s="7">
         <v>62</v>
       </c>
+      <c r="CN5" s="7">
+        <v>25</v>
+      </c>
     </row>
-    <row r="6" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" s="9">
         <v>2</v>
@@ -28848,10 +29149,13 @@
       <c r="CM6" s="9">
         <v>0</v>
       </c>
+      <c r="CN6" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B7" s="10">
         <v>4</v>
@@ -29123,10 +29427,13 @@
       <c r="CM7" s="10">
         <v>0</v>
       </c>
+      <c r="CN7" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B8" s="9">
         <v>3</v>
@@ -29398,10 +29705,13 @@
       <c r="CM8" s="9">
         <v>0</v>
       </c>
+      <c r="CN8" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B9" s="10">
         <v>6</v>
@@ -29673,10 +29983,13 @@
       <c r="CM9" s="10">
         <v>0</v>
       </c>
+      <c r="CN9" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" s="9">
         <v>8</v>
@@ -29948,10 +30261,13 @@
       <c r="CM10" s="9">
         <v>0</v>
       </c>
+      <c r="CN10" s="9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B11" s="10">
         <v>5</v>
@@ -30223,10 +30539,13 @@
       <c r="CM11" s="10">
         <v>0</v>
       </c>
+      <c r="CN11" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B12" s="9">
         <v>1</v>
@@ -30498,10 +30817,13 @@
       <c r="CM12" s="9">
         <v>0</v>
       </c>
+      <c r="CN12" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B13" s="10">
         <v>4</v>
@@ -30773,10 +31095,13 @@
       <c r="CM13" s="10">
         <v>0</v>
       </c>
+      <c r="CN13" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14" s="9">
         <v>3</v>
@@ -31048,10 +31373,13 @@
       <c r="CM14" s="9">
         <v>0</v>
       </c>
+      <c r="CN14" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B15" s="10">
         <v>330</v>
@@ -31323,10 +31651,13 @@
       <c r="CM15" s="10">
         <v>1</v>
       </c>
+      <c r="CN15" s="10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="16" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="9">
         <v>2</v>
@@ -31598,10 +31929,13 @@
       <c r="CM16" s="9">
         <v>0</v>
       </c>
+      <c r="CN16" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" s="10">
         <v>3</v>
@@ -31873,10 +32207,13 @@
       <c r="CM17" s="10">
         <v>0</v>
       </c>
+      <c r="CN17" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B18" s="9">
         <v>7</v>
@@ -32148,10 +32485,13 @@
       <c r="CM18" s="9">
         <v>0</v>
       </c>
+      <c r="CN18" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B19" s="10">
         <v>5</v>
@@ -32423,10 +32763,13 @@
       <c r="CM19" s="10">
         <v>0</v>
       </c>
+      <c r="CN19" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B20" s="9">
         <v>3</v>
@@ -32698,10 +33041,13 @@
       <c r="CM20" s="9">
         <v>0</v>
       </c>
+      <c r="CN20" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" s="10">
         <v>6</v>
@@ -32973,10 +33319,13 @@
       <c r="CM21" s="10">
         <v>0</v>
       </c>
+      <c r="CN21" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B22" s="9">
         <v>4</v>
@@ -33248,10 +33597,13 @@
       <c r="CM22" s="9">
         <v>0</v>
       </c>
+      <c r="CN22" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B23" s="10">
         <v>2356</v>
@@ -33523,10 +33875,13 @@
       <c r="CM23" s="10">
         <v>60</v>
       </c>
+      <c r="CN23" s="10">
+        <v>23</v>
+      </c>
     </row>
-    <row r="24" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B24" s="11">
         <v>936</v>
@@ -33798,10 +34153,13 @@
       <c r="CM24" s="11">
         <v>5</v>
       </c>
+      <c r="CN24" s="11">
+        <v>2</v>
+      </c>
     </row>
-    <row r="25" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B25" s="10">
         <v>3</v>
@@ -34073,10 +34431,13 @@
       <c r="CM25" s="10">
         <v>0</v>
       </c>
+      <c r="CN25" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B26" s="9">
         <v>1</v>
@@ -34348,10 +34709,13 @@
       <c r="CM26" s="9">
         <v>0</v>
       </c>
+      <c r="CN26" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B27" s="10">
         <v>2</v>
@@ -34623,10 +34987,13 @@
       <c r="CM27" s="10">
         <v>0</v>
       </c>
+      <c r="CN27" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B28" s="9">
         <v>0</v>
@@ -34898,10 +35265,13 @@
       <c r="CM28" s="9">
         <v>0</v>
       </c>
+      <c r="CN28" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="29" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B29" s="10">
         <v>2</v>
@@ -35173,10 +35543,13 @@
       <c r="CM29" s="10">
         <v>0</v>
       </c>
+      <c r="CN29" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B30" s="9">
         <v>3</v>
@@ -35448,10 +35821,13 @@
       <c r="CM30" s="9">
         <v>0</v>
       </c>
+      <c r="CN30" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B31" s="10">
         <v>11</v>
@@ -35723,10 +36099,13 @@
       <c r="CM31" s="10">
         <v>0</v>
       </c>
+      <c r="CN31" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="32" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B32" s="9">
         <v>14</v>
@@ -35998,10 +36377,13 @@
       <c r="CM32" s="9">
         <v>1</v>
       </c>
+      <c r="CN32" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B33" s="10">
         <v>2</v>
@@ -36273,10 +36655,13 @@
       <c r="CM33" s="10">
         <v>0</v>
       </c>
+      <c r="CN33" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B34" s="9">
         <v>3</v>
@@ -36548,10 +36933,13 @@
       <c r="CM34" s="9">
         <v>0</v>
       </c>
+      <c r="CN34" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="35" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" s="10">
         <v>0</v>
@@ -36823,10 +37211,13 @@
       <c r="CM35" s="10">
         <v>0</v>
       </c>
+      <c r="CN35" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="36" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B36" s="9">
         <v>899</v>
@@ -37098,10 +37489,13 @@
       <c r="CM36" s="9">
         <v>4</v>
       </c>
+      <c r="CN36" s="9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="37" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B37" s="7">
         <v>50</v>
@@ -37373,10 +37767,13 @@
       <c r="CM37" s="7">
         <v>0</v>
       </c>
+      <c r="CN37" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="38" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B38" s="9">
         <v>0</v>
@@ -37648,10 +38045,13 @@
       <c r="CM38" s="9">
         <v>0</v>
       </c>
+      <c r="CN38" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B39" s="10">
         <v>0</v>
@@ -37923,10 +38323,13 @@
       <c r="CM39" s="10">
         <v>0</v>
       </c>
+      <c r="CN39" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B40" s="9">
         <v>1</v>
@@ -38198,10 +38601,13 @@
       <c r="CM40" s="9">
         <v>0</v>
       </c>
+      <c r="CN40" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="41" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B41" s="10">
         <v>25</v>
@@ -38473,10 +38879,13 @@
       <c r="CM41" s="10">
         <v>0</v>
       </c>
+      <c r="CN41" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B42" s="9">
         <v>2</v>
@@ -38748,10 +39157,13 @@
       <c r="CM42" s="9">
         <v>0</v>
       </c>
+      <c r="CN42" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B43" s="10">
         <v>4</v>
@@ -39023,10 +39435,13 @@
       <c r="CM43" s="10">
         <v>0</v>
       </c>
+      <c r="CN43" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B44" s="9">
         <v>17</v>
@@ -39298,10 +39713,13 @@
       <c r="CM44" s="9">
         <v>0</v>
       </c>
+      <c r="CN44" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B45" s="10">
         <v>0</v>
@@ -39573,10 +39991,13 @@
       <c r="CM45" s="10">
         <v>0</v>
       </c>
+      <c r="CN45" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B46" s="11">
         <v>23</v>
@@ -39848,10 +40269,13 @@
       <c r="CM46" s="11">
         <v>1</v>
       </c>
+      <c r="CN46" s="11">
+        <v>1</v>
+      </c>
     </row>
-    <row r="47" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B47" s="10">
         <v>10</v>
@@ -40123,10 +40547,13 @@
       <c r="CM47" s="10">
         <v>0</v>
       </c>
+      <c r="CN47" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="48" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B48" s="9">
         <v>0</v>
@@ -40398,10 +40825,13 @@
       <c r="CM48" s="9">
         <v>0</v>
       </c>
+      <c r="CN48" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="49" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B49" s="10">
         <v>1</v>
@@ -40673,10 +41103,13 @@
       <c r="CM49" s="10">
         <v>0</v>
       </c>
+      <c r="CN49" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="50" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B50" s="9">
         <v>0</v>
@@ -40948,10 +41381,13 @@
       <c r="CM50" s="9">
         <v>0</v>
       </c>
+      <c r="CN50" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="51" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B51" s="10">
         <v>4</v>
@@ -41223,10 +41659,13 @@
       <c r="CM51" s="10">
         <v>0</v>
       </c>
+      <c r="CN51" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="52" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B52" s="9">
         <v>1</v>
@@ -41498,10 +41937,13 @@
       <c r="CM52" s="9">
         <v>0</v>
       </c>
+      <c r="CN52" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="53" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B53" s="10">
         <v>7</v>
@@ -41773,10 +42215,13 @@
       <c r="CM53" s="10">
         <v>1</v>
       </c>
+      <c r="CN53" s="10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="54" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B54" s="11">
         <v>89</v>
@@ -42048,10 +42493,13 @@
       <c r="CM54" s="11">
         <v>1</v>
       </c>
+      <c r="CN54" s="11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="55" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B55" s="10">
         <v>10</v>
@@ -42323,10 +42771,13 @@
       <c r="CM55" s="10">
         <v>0</v>
       </c>
+      <c r="CN55" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="56" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B56" s="9">
         <v>0</v>
@@ -42598,10 +43049,13 @@
       <c r="CM56" s="9">
         <v>0</v>
       </c>
+      <c r="CN56" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="57" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B57" s="10">
         <v>1</v>
@@ -42873,10 +43327,13 @@
       <c r="CM57" s="10">
         <v>0</v>
       </c>
+      <c r="CN57" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="58" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B58" s="9">
         <v>10</v>
@@ -43148,10 +43605,13 @@
       <c r="CM58" s="9">
         <v>0</v>
       </c>
+      <c r="CN58" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="59" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B59" s="10">
         <v>4</v>
@@ -43423,10 +43883,13 @@
       <c r="CM59" s="10">
         <v>0</v>
       </c>
+      <c r="CN59" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="60" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B60" s="9">
         <v>8</v>
@@ -43698,10 +44161,13 @@
       <c r="CM60" s="9">
         <v>0</v>
       </c>
+      <c r="CN60" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="61" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B61" s="10">
         <v>15</v>
@@ -43973,10 +44439,13 @@
       <c r="CM61" s="10">
         <v>1</v>
       </c>
+      <c r="CN61" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="62" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B62" s="9">
         <v>4</v>
@@ -44248,10 +44717,13 @@
       <c r="CM62" s="9">
         <v>0</v>
       </c>
+      <c r="CN62" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="63" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B63" s="10">
         <v>12</v>
@@ -44523,10 +44995,13 @@
       <c r="CM63" s="10">
         <v>0</v>
       </c>
+      <c r="CN63" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="64" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B64" s="9">
         <v>3</v>
@@ -44798,10 +45273,13 @@
       <c r="CM64" s="9">
         <v>0</v>
       </c>
+      <c r="CN64" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="65" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B65" s="10">
         <v>2</v>
@@ -45073,10 +45551,13 @@
       <c r="CM65" s="10">
         <v>0</v>
       </c>
+      <c r="CN65" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="66" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" s="9">
         <v>10</v>
@@ -45348,10 +45829,13 @@
       <c r="CM66" s="9">
         <v>0</v>
       </c>
+      <c r="CN66" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="67" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B67" s="10">
         <v>6</v>
@@ -45623,10 +46107,13 @@
       <c r="CM67" s="10">
         <v>0</v>
       </c>
+      <c r="CN67" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="68" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B68" s="9">
         <v>4</v>
@@ -45898,10 +46385,13 @@
       <c r="CM68" s="9">
         <v>0</v>
       </c>
+      <c r="CN68" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="69" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B69" s="7">
         <v>45</v>
@@ -46173,10 +46663,13 @@
       <c r="CM69" s="7">
         <v>0</v>
       </c>
+      <c r="CN69" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="70" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="9">
         <v>1</v>
@@ -46448,10 +46941,13 @@
       <c r="CM70" s="9">
         <v>0</v>
       </c>
+      <c r="CN70" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="71" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B71" s="10">
         <v>23</v>
@@ -46723,10 +47219,13 @@
       <c r="CM71" s="10">
         <v>0</v>
       </c>
+      <c r="CN71" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="72" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B72" s="9">
         <v>7</v>
@@ -46998,10 +47497,13 @@
       <c r="CM72" s="9">
         <v>0</v>
       </c>
+      <c r="CN72" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="73" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B73" s="10">
         <v>2</v>
@@ -47273,10 +47775,13 @@
       <c r="CM73" s="10">
         <v>0</v>
       </c>
+      <c r="CN73" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="74" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B74" s="9">
         <v>1</v>
@@ -47548,10 +48053,13 @@
       <c r="CM74" s="9">
         <v>0</v>
       </c>
+      <c r="CN74" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="75" spans="1:91" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:92" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B75" s="10">
         <v>4</v>
@@ -47823,10 +48331,13 @@
       <c r="CM75" s="10">
         <v>0</v>
       </c>
+      <c r="CN75" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="76" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B76" s="9">
         <v>14</v>
@@ -48098,10 +48609,13 @@
       <c r="CM76" s="9">
         <v>0</v>
       </c>
+      <c r="CN76" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="77" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B77" s="7">
         <v>63</v>
@@ -48373,10 +48887,13 @@
       <c r="CM77" s="7">
         <v>1</v>
       </c>
+      <c r="CN77" s="7">
+        <v>2</v>
+      </c>
     </row>
-    <row r="78" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B78" s="9">
         <v>0</v>
@@ -48648,10 +49165,13 @@
       <c r="CM78" s="9">
         <v>0</v>
       </c>
+      <c r="CN78" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="79" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B79" s="10">
         <v>0</v>
@@ -48923,10 +49443,13 @@
       <c r="CM79" s="10">
         <v>0</v>
       </c>
+      <c r="CN79" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="80" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B80" s="9">
         <v>0</v>
@@ -49198,10 +49721,13 @@
       <c r="CM80" s="9">
         <v>0</v>
       </c>
+      <c r="CN80" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="81" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B81" s="10">
         <v>5</v>
@@ -49473,10 +49999,13 @@
       <c r="CM81" s="10">
         <v>0</v>
       </c>
+      <c r="CN81" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="82" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B82" s="9">
         <v>19</v>
@@ -49748,10 +50277,13 @@
       <c r="CM82" s="9">
         <v>1</v>
       </c>
+      <c r="CN82" s="9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="83" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B83" s="10">
         <v>4</v>
@@ -50023,10 +50555,13 @@
       <c r="CM83" s="10">
         <v>0</v>
       </c>
+      <c r="CN83" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="84" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B84" s="9">
         <v>4</v>
@@ -50298,10 +50833,13 @@
       <c r="CM84" s="9">
         <v>0</v>
       </c>
+      <c r="CN84" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="85" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B85" s="10">
         <v>20</v>
@@ -50573,10 +51111,13 @@
       <c r="CM85" s="10">
         <v>0</v>
       </c>
+      <c r="CN85" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="86" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B86" s="9">
         <v>9</v>
@@ -50848,10 +51389,13 @@
       <c r="CM86" s="9">
         <v>0</v>
       </c>
+      <c r="CN86" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="87" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B87" s="10">
         <v>2</v>
@@ -51123,10 +51667,13 @@
       <c r="CM87" s="10">
         <v>0</v>
       </c>
+      <c r="CN87" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="88" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B88" s="11">
         <v>31</v>
@@ -51398,10 +51945,13 @@
       <c r="CM88" s="11">
         <v>0</v>
       </c>
+      <c r="CN88" s="11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="89" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B89" s="10">
         <v>1</v>
@@ -51673,10 +52223,13 @@
       <c r="CM89" s="10">
         <v>0</v>
       </c>
+      <c r="CN89" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="90" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B90" s="9">
         <v>2</v>
@@ -51948,10 +52501,13 @@
       <c r="CM90" s="9">
         <v>0</v>
       </c>
+      <c r="CN90" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="91" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B91" s="10">
         <v>2</v>
@@ -52223,10 +52779,13 @@
       <c r="CM91" s="10">
         <v>0</v>
       </c>
+      <c r="CN91" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="92" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B92" s="9">
         <v>1</v>
@@ -52498,10 +53057,13 @@
       <c r="CM92" s="9">
         <v>0</v>
       </c>
+      <c r="CN92" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="93" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B93" s="10">
         <v>21</v>
@@ -52773,10 +53335,13 @@
       <c r="CM93" s="10">
         <v>0</v>
       </c>
+      <c r="CN93" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="94" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B94" s="9">
         <v>3</v>
@@ -53048,10 +53613,13 @@
       <c r="CM94" s="9">
         <v>0</v>
       </c>
+      <c r="CN94" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="95" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B95" s="10">
         <v>0</v>
@@ -53323,10 +53891,13 @@
       <c r="CM95" s="10">
         <v>0</v>
       </c>
+      <c r="CN95" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="96" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B96" s="9">
         <v>0</v>
@@ -53598,10 +54169,13 @@
       <c r="CM96" s="9">
         <v>0</v>
       </c>
+      <c r="CN96" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="97" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B97" s="10">
         <v>0</v>
@@ -53873,10 +54447,13 @@
       <c r="CM97" s="10">
         <v>0</v>
       </c>
+      <c r="CN97" s="10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="98" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B98" s="9">
         <v>0</v>
@@ -54148,10 +54725,13 @@
       <c r="CM98" s="9">
         <v>0</v>
       </c>
+      <c r="CN98" s="9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="99" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B99" s="10">
         <v>0</v>
@@ -54421,6 +55001,9 @@
         <v>0</v>
       </c>
       <c r="CM99" s="10">
+        <v>0</v>
+      </c>
+      <c r="CN99" s="10">
         <v>0</v>
       </c>
     </row>
@@ -54436,18 +55019,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Лист3"/>
-  <dimension ref="A1:CM99"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:CN99"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.85546875" customWidth="1"/>
-    <col min="2" max="91" width="16.7109375" customWidth="1"/>
+    <col min="2" max="92" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:91" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:91" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:92" s="1" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:92" s="1" customFormat="1" ht="44.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -54463,7 +55045,7 @@
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
     </row>
-    <row r="3" spans="1:91" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:92" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>0</v>
@@ -54735,10 +55317,13 @@
       <c r="CM3" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="CN3" s="3" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="5">
         <v>901825</v>
@@ -55010,10 +55595,13 @@
       <c r="CM4" s="5">
         <v>2362978</v>
       </c>
+      <c r="CN4" s="5">
+        <v>2278577</v>
+      </c>
     </row>
-    <row r="5" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="7">
         <v>294911</v>
@@ -55285,10 +55873,13 @@
       <c r="CM5" s="7">
         <v>740566</v>
       </c>
+      <c r="CN5" s="7">
+        <v>711293</v>
+      </c>
     </row>
-    <row r="6" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" s="9">
         <v>7772</v>
@@ -55560,10 +56151,13 @@
       <c r="CM6" s="9">
         <v>20553</v>
       </c>
+      <c r="CN6" s="9">
+        <v>19350</v>
+      </c>
     </row>
-    <row r="7" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B7" s="10">
         <v>5107</v>
@@ -55835,10 +56429,13 @@
       <c r="CM7" s="10">
         <v>13724</v>
       </c>
+      <c r="CN7" s="10">
+        <v>13631</v>
+      </c>
     </row>
-    <row r="8" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B8" s="9">
         <v>6198</v>
@@ -56110,10 +56707,13 @@
       <c r="CM8" s="9">
         <v>17299</v>
       </c>
+      <c r="CN8" s="9">
+        <v>16889</v>
+      </c>
     </row>
-    <row r="9" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B9" s="10">
         <v>11670</v>
@@ -56385,10 +56985,13 @@
       <c r="CM9" s="10">
         <v>31613</v>
       </c>
+      <c r="CN9" s="10">
+        <v>29377</v>
+      </c>
     </row>
-    <row r="10" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" s="9">
         <v>4159</v>
@@ -56660,10 +57263,13 @@
       <c r="CM10" s="9">
         <v>11403</v>
       </c>
+      <c r="CN10" s="9">
+        <v>10844</v>
+      </c>
     </row>
-    <row r="11" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B11" s="10">
         <v>6335</v>
@@ -56935,10 +57541,13 @@
       <c r="CM11" s="10">
         <v>16134</v>
       </c>
+      <c r="CN11" s="10">
+        <v>15609</v>
+      </c>
     </row>
-    <row r="12" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B12" s="9">
         <v>2781</v>
@@ -57210,10 +57819,13 @@
       <c r="CM12" s="9">
         <v>7878</v>
       </c>
+      <c r="CN12" s="9">
+        <v>7056</v>
+      </c>
     </row>
-    <row r="13" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B13" s="10">
         <v>5467</v>
@@ -57485,10 +58097,13 @@
       <c r="CM13" s="10">
         <v>13763</v>
       </c>
+      <c r="CN13" s="10">
+        <v>13299</v>
+      </c>
     </row>
-    <row r="14" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14" s="9">
         <v>5960</v>
@@ -57760,10 +58375,13 @@
       <c r="CM14" s="9">
         <v>14588</v>
       </c>
+      <c r="CN14" s="9">
+        <v>13939</v>
+      </c>
     </row>
-    <row r="15" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B15" s="10">
         <v>70420</v>
@@ -58035,10 +58653,13 @@
       <c r="CM15" s="10">
         <v>188123</v>
       </c>
+      <c r="CN15" s="10">
+        <v>178746</v>
+      </c>
     </row>
-    <row r="16" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="9">
         <v>3847</v>
@@ -58310,10 +58931,13 @@
       <c r="CM16" s="9">
         <v>9110</v>
       </c>
+      <c r="CN16" s="9">
+        <v>8987</v>
+      </c>
     </row>
-    <row r="17" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" s="10">
         <v>5627</v>
@@ -58585,10 +59209,13 @@
       <c r="CM17" s="10">
         <v>15344</v>
       </c>
+      <c r="CN17" s="10">
+        <v>14531</v>
+      </c>
     </row>
-    <row r="18" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B18" s="9">
         <v>4674</v>
@@ -58860,10 +59487,13 @@
       <c r="CM18" s="9">
         <v>11674</v>
       </c>
+      <c r="CN18" s="9">
+        <v>11679</v>
+      </c>
     </row>
-    <row r="19" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B19" s="10">
         <v>4641</v>
@@ -59135,10 +59765,13 @@
       <c r="CM19" s="10">
         <v>10808</v>
       </c>
+      <c r="CN19" s="10">
+        <v>10399</v>
+      </c>
     </row>
-    <row r="20" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B20" s="9">
         <v>6902</v>
@@ -59410,10 +60043,13 @@
       <c r="CM20" s="9">
         <v>16784</v>
       </c>
+      <c r="CN20" s="9">
+        <v>16569</v>
+      </c>
     </row>
-    <row r="21" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" s="10">
         <v>8410</v>
@@ -59685,10 +60321,13 @@
       <c r="CM21" s="10">
         <v>21068</v>
       </c>
+      <c r="CN21" s="10">
+        <v>20132</v>
+      </c>
     </row>
-    <row r="22" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B22" s="9">
         <v>6156</v>
@@ -59960,10 +60599,13 @@
       <c r="CM22" s="9">
         <v>17038</v>
       </c>
+      <c r="CN22" s="9">
+        <v>16140</v>
+      </c>
     </row>
-    <row r="23" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B23" s="10">
         <v>128782</v>
@@ -60235,10 +60877,13 @@
       <c r="CM23" s="10">
         <v>303662</v>
       </c>
+      <c r="CN23" s="10">
+        <v>294117</v>
+      </c>
     </row>
-    <row r="24" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B24" s="11">
         <v>112892</v>
@@ -60510,10 +61155,13 @@
       <c r="CM24" s="11">
         <v>269454</v>
       </c>
+      <c r="CN24" s="11">
+        <v>258592</v>
+      </c>
     </row>
-    <row r="25" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B25" s="10">
         <v>4101</v>
@@ -60785,10 +61433,13 @@
       <c r="CM25" s="10">
         <v>9323</v>
       </c>
+      <c r="CN25" s="10">
+        <v>9029</v>
+      </c>
     </row>
-    <row r="26" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B26" s="9">
         <v>6270</v>
@@ -61060,10 +61711,13 @@
       <c r="CM26" s="9">
         <v>12862</v>
       </c>
+      <c r="CN26" s="9">
+        <v>12604</v>
+      </c>
     </row>
-    <row r="27" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B27" s="10">
         <v>7905</v>
@@ -61335,10 +61989,13 @@
       <c r="CM27" s="10">
         <v>18182</v>
       </c>
+      <c r="CN27" s="10">
+        <v>18236</v>
+      </c>
     </row>
-    <row r="28" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B28" s="9">
         <v>360</v>
@@ -61610,10 +62267,13 @@
       <c r="CM28" s="9">
         <v>768</v>
       </c>
+      <c r="CN28" s="9">
+        <v>891</v>
+      </c>
     </row>
-    <row r="29" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B29" s="10">
         <v>7545</v>
@@ -61885,10 +62545,13 @@
       <c r="CM29" s="10">
         <v>17415</v>
       </c>
+      <c r="CN29" s="10">
+        <v>17345</v>
+      </c>
     </row>
-    <row r="30" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B30" s="9">
         <v>6487</v>
@@ -62160,10 +62823,13 @@
       <c r="CM30" s="9">
         <v>16910</v>
       </c>
+      <c r="CN30" s="9">
+        <v>15903</v>
+      </c>
     </row>
-    <row r="31" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B31" s="10">
         <v>6729</v>
@@ -62435,10 +63101,13 @@
       <c r="CM31" s="10">
         <v>18883</v>
       </c>
+      <c r="CN31" s="10">
+        <v>18577</v>
+      </c>
     </row>
-    <row r="32" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B32" s="9">
         <v>13510</v>
@@ -62710,10 +63379,13 @@
       <c r="CM32" s="9">
         <v>36654</v>
       </c>
+      <c r="CN32" s="9">
+        <v>35107</v>
+      </c>
     </row>
-    <row r="33" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B33" s="10">
         <v>6788</v>
@@ -62985,10 +63657,13 @@
       <c r="CM33" s="10">
         <v>14246</v>
       </c>
+      <c r="CN33" s="10">
+        <v>14112</v>
+      </c>
     </row>
-    <row r="34" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B34" s="9">
         <v>3076</v>
@@ -63260,10 +63935,13 @@
       <c r="CM34" s="9">
         <v>7939</v>
       </c>
+      <c r="CN34" s="9">
+        <v>7489</v>
+      </c>
     </row>
-    <row r="35" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" s="10">
         <v>2981</v>
@@ -63535,10 +64213,13 @@
       <c r="CM35" s="10">
         <v>7657</v>
       </c>
+      <c r="CN35" s="10">
+        <v>7443</v>
+      </c>
     </row>
-    <row r="36" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B36" s="9">
         <v>55043</v>
@@ -63810,10 +64491,13 @@
       <c r="CM36" s="9">
         <v>126796</v>
       </c>
+      <c r="CN36" s="9">
+        <v>120093</v>
+      </c>
     </row>
-    <row r="37" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B37" s="7">
         <v>73845</v>
@@ -64085,10 +64769,13 @@
       <c r="CM37" s="7">
         <v>231571</v>
       </c>
+      <c r="CN37" s="7">
+        <v>221718</v>
+      </c>
     </row>
-    <row r="38" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B38" s="9">
         <v>1931</v>
@@ -64360,10 +65047,13 @@
       <c r="CM38" s="9">
         <v>5921</v>
       </c>
+      <c r="CN38" s="9">
+        <v>6037</v>
+      </c>
     </row>
-    <row r="39" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B39" s="10">
         <v>1585</v>
@@ -64635,10 +65325,13 @@
       <c r="CM39" s="10">
         <v>5397</v>
       </c>
+      <c r="CN39" s="10">
+        <v>5225</v>
+      </c>
     </row>
-    <row r="40" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B40" s="9">
         <v>1598</v>
@@ -64910,10 +65603,13 @@
       <c r="CM40" s="9">
         <v>19537</v>
       </c>
+      <c r="CN40" s="9">
+        <v>17010</v>
+      </c>
     </row>
-    <row r="41" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B41" s="10">
         <v>30789</v>
@@ -65185,10 +65881,13 @@
       <c r="CM41" s="10">
         <v>92003</v>
       </c>
+      <c r="CN41" s="10">
+        <v>88449</v>
+      </c>
     </row>
-    <row r="42" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B42" s="9">
         <v>5007</v>
@@ -65460,10 +66159,13 @@
       <c r="CM42" s="9">
         <v>13437</v>
       </c>
+      <c r="CN42" s="9">
+        <v>13013</v>
+      </c>
     </row>
-    <row r="43" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B43" s="10">
         <v>11916</v>
@@ -65735,10 +66437,13 @@
       <c r="CM43" s="10">
         <v>29608</v>
       </c>
+      <c r="CN43" s="10">
+        <v>28683</v>
+      </c>
     </row>
-    <row r="44" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B44" s="9">
         <v>20505</v>
@@ -66010,10 +66715,13 @@
       <c r="CM44" s="9">
         <v>59887</v>
       </c>
+      <c r="CN44" s="9">
+        <v>57773</v>
+      </c>
     </row>
-    <row r="45" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B45" s="10">
         <v>514</v>
@@ -66285,10 +66993,13 @@
       <c r="CM45" s="10">
         <v>5781</v>
       </c>
+      <c r="CN45" s="10">
+        <v>5520</v>
+      </c>
     </row>
-    <row r="46" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B46" s="11">
         <v>22881</v>
@@ -66560,10 +67271,13 @@
       <c r="CM46" s="11">
         <v>65653</v>
       </c>
+      <c r="CN46" s="11">
+        <v>64103</v>
+      </c>
     </row>
-    <row r="47" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B47" s="10">
         <v>3036</v>
@@ -66835,10 +67549,13 @@
       <c r="CM47" s="10">
         <v>11152</v>
       </c>
+      <c r="CN47" s="10">
+        <v>10793</v>
+      </c>
     </row>
-    <row r="48" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B48" s="9">
         <v>317</v>
@@ -67110,10 +67827,13 @@
       <c r="CM48" s="9">
         <v>1068</v>
       </c>
+      <c r="CN48" s="9">
+        <v>1111</v>
+      </c>
     </row>
-    <row r="49" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B49" s="10">
         <v>2002</v>
@@ -67385,10 +68105,13 @@
       <c r="CM49" s="10">
         <v>5718</v>
       </c>
+      <c r="CN49" s="10">
+        <v>5825</v>
+      </c>
     </row>
-    <row r="50" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B50" s="9">
         <v>1368</v>
@@ -67660,10 +68383,13 @@
       <c r="CM50" s="9">
         <v>3923</v>
       </c>
+      <c r="CN50" s="9">
+        <v>3939</v>
+      </c>
     </row>
-    <row r="51" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B51" s="10">
         <v>2390</v>
@@ -67935,10 +68661,13 @@
       <c r="CM51" s="10">
         <v>6378</v>
       </c>
+      <c r="CN51" s="10">
+        <v>6371</v>
+      </c>
     </row>
-    <row r="52" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B52" s="9">
         <v>1219</v>
@@ -68210,10 +68939,13 @@
       <c r="CM52" s="9">
         <v>4523</v>
       </c>
+      <c r="CN52" s="9">
+        <v>4664</v>
+      </c>
     </row>
-    <row r="53" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B53" s="10">
         <v>12550</v>
@@ -68485,10 +69217,13 @@
       <c r="CM53" s="10">
         <v>32891</v>
       </c>
+      <c r="CN53" s="10">
+        <v>31402</v>
+      </c>
     </row>
-    <row r="54" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B54" s="11">
         <v>157685</v>
@@ -68760,10 +69495,13 @@
       <c r="CM54" s="11">
         <v>433794</v>
       </c>
+      <c r="CN54" s="11">
+        <v>416041</v>
+      </c>
     </row>
-    <row r="55" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B55" s="10">
         <v>22879</v>
@@ -69035,10 +69773,13 @@
       <c r="CM55" s="10">
         <v>62849</v>
       </c>
+      <c r="CN55" s="10">
+        <v>58894</v>
+      </c>
     </row>
-    <row r="56" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B56" s="9">
         <v>3119</v>
@@ -69310,10 +70051,13 @@
       <c r="CM56" s="9">
         <v>8998</v>
       </c>
+      <c r="CN56" s="9">
+        <v>8234</v>
+      </c>
     </row>
-    <row r="57" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B57" s="10">
         <v>3238</v>
@@ -69585,10 +70329,13 @@
       <c r="CM57" s="10">
         <v>8893</v>
       </c>
+      <c r="CN57" s="10">
+        <v>8660</v>
+      </c>
     </row>
-    <row r="58" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B58" s="9">
         <v>23250</v>
@@ -69860,10 +70607,13 @@
       <c r="CM58" s="9">
         <v>67429</v>
       </c>
+      <c r="CN58" s="9">
+        <v>64240</v>
+      </c>
     </row>
-    <row r="59" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B59" s="10">
         <v>8601</v>
@@ -70135,10 +70885,13 @@
       <c r="CM59" s="10">
         <v>25619</v>
       </c>
+      <c r="CN59" s="10">
+        <v>23973</v>
+      </c>
     </row>
-    <row r="60" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B60" s="9">
         <v>6292</v>
@@ -70410,10 +71163,13 @@
       <c r="CM60" s="9">
         <v>17731</v>
       </c>
+      <c r="CN60" s="9">
+        <v>17012</v>
+      </c>
     </row>
-    <row r="61" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B61" s="10">
         <v>16320</v>
@@ -70685,10 +71441,13 @@
       <c r="CM61" s="10">
         <v>43928</v>
       </c>
+      <c r="CN61" s="10">
+        <v>41349</v>
+      </c>
     </row>
-    <row r="62" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B62" s="9">
         <v>6207</v>
@@ -70960,10 +71719,13 @@
       <c r="CM62" s="9">
         <v>17349</v>
       </c>
+      <c r="CN62" s="9">
+        <v>16324</v>
+      </c>
     </row>
-    <row r="63" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B63" s="10">
         <v>16527</v>
@@ -71235,10 +71997,13 @@
       <c r="CM63" s="10">
         <v>47522</v>
       </c>
+      <c r="CN63" s="10">
+        <v>45953</v>
+      </c>
     </row>
-    <row r="64" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B64" s="9">
         <v>10594</v>
@@ -71510,10 +72275,13 @@
       <c r="CM64" s="9">
         <v>28042</v>
       </c>
+      <c r="CN64" s="9">
+        <v>27661</v>
+      </c>
     </row>
-    <row r="65" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B65" s="10">
         <v>5922</v>
@@ -71785,10 +72553,13 @@
       <c r="CM65" s="10">
         <v>15367</v>
       </c>
+      <c r="CN65" s="10">
+        <v>14660</v>
+      </c>
     </row>
-    <row r="66" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" s="9">
         <v>18073</v>
@@ -72060,10 +72831,13 @@
       <c r="CM66" s="9">
         <v>45975</v>
       </c>
+      <c r="CN66" s="9">
+        <v>45757</v>
+      </c>
     </row>
-    <row r="67" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B67" s="10">
         <v>10810</v>
@@ -72335,10 +73109,13 @@
       <c r="CM67" s="10">
         <v>29387</v>
       </c>
+      <c r="CN67" s="10">
+        <v>28583</v>
+      </c>
     </row>
-    <row r="68" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B68" s="9">
         <v>5853</v>
@@ -72610,10 +73387,13 @@
       <c r="CM68" s="9">
         <v>14705</v>
       </c>
+      <c r="CN68" s="9">
+        <v>14740</v>
+      </c>
     </row>
-    <row r="69" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B69" s="7">
         <v>88686</v>
@@ -72885,10 +73665,13 @@
       <c r="CM69" s="7">
         <v>226369</v>
       </c>
+      <c r="CN69" s="7">
+        <v>217760</v>
+      </c>
     </row>
-    <row r="70" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="9">
         <v>4082</v>
@@ -73160,10 +73943,13 @@
       <c r="CM70" s="9">
         <v>10747</v>
       </c>
+      <c r="CN70" s="9">
+        <v>10599</v>
+      </c>
     </row>
-    <row r="71" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B71" s="10">
         <v>28809</v>
@@ -73435,10 +74221,13 @@
       <c r="CM71" s="10">
         <v>75048</v>
       </c>
+      <c r="CN71" s="10">
+        <v>72133</v>
+      </c>
     </row>
-    <row r="72" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B72" s="9">
         <v>36580</v>
@@ -73710,10 +74499,13 @@
       <c r="CM72" s="9">
         <v>87097</v>
       </c>
+      <c r="CN72" s="9">
+        <v>83773</v>
+      </c>
     </row>
-    <row r="73" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B73" s="10">
         <v>16942</v>
@@ -73985,10 +74777,13 @@
       <c r="CM73" s="10">
         <v>36358</v>
       </c>
+      <c r="CN73" s="10">
+        <v>35659</v>
+      </c>
     </row>
-    <row r="74" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B74" s="9">
         <v>5986</v>
@@ -74260,10 +75055,13 @@
       <c r="CM74" s="9">
         <v>14219</v>
       </c>
+      <c r="CN74" s="9">
+        <v>14277</v>
+      </c>
     </row>
-    <row r="75" spans="1:91" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:92" s="1" customFormat="1" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B75" s="10">
         <v>13652</v>
@@ -74535,10 +75333,13 @@
       <c r="CM75" s="10">
         <v>36520</v>
       </c>
+      <c r="CN75" s="10">
+        <v>33836</v>
+      </c>
     </row>
-    <row r="76" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B76" s="9">
         <v>19216</v>
@@ -74810,10 +75611,13 @@
       <c r="CM76" s="9">
         <v>53477</v>
       </c>
+      <c r="CN76" s="9">
+        <v>51256</v>
+      </c>
     </row>
-    <row r="77" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B77" s="7">
         <v>98327</v>
@@ -75085,10 +75889,13 @@
       <c r="CM77" s="7">
         <v>260703</v>
       </c>
+      <c r="CN77" s="7">
+        <v>253395</v>
+      </c>
     </row>
-    <row r="78" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B78" s="9">
         <v>921</v>
@@ -75360,10 +76167,13 @@
       <c r="CM78" s="9">
         <v>3307</v>
       </c>
+      <c r="CN78" s="9">
+        <v>3326</v>
+      </c>
     </row>
-    <row r="79" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B79" s="10">
         <v>1461</v>
@@ -75635,10 +76445,13 @@
       <c r="CM79" s="10">
         <v>5398</v>
       </c>
+      <c r="CN79" s="10">
+        <v>5375</v>
+      </c>
     </row>
-    <row r="80" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B80" s="9">
         <v>2551</v>
@@ -75910,10 +76723,13 @@
       <c r="CM80" s="9">
         <v>7938</v>
       </c>
+      <c r="CN80" s="9">
+        <v>7919</v>
+      </c>
     </row>
-    <row r="81" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B81" s="10">
         <v>10659</v>
@@ -76185,10 +77001,13 @@
       <c r="CM81" s="10">
         <v>27857</v>
       </c>
+      <c r="CN81" s="10">
+        <v>26958</v>
+      </c>
     </row>
-    <row r="82" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B82" s="9">
         <v>17861</v>
@@ -76460,10 +77279,13 @@
       <c r="CM82" s="9">
         <v>47576</v>
       </c>
+      <c r="CN82" s="9">
+        <v>46531</v>
+      </c>
     </row>
-    <row r="83" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B83" s="10">
         <v>14677</v>
@@ -76735,10 +77557,13 @@
       <c r="CM83" s="10">
         <v>38299</v>
       </c>
+      <c r="CN83" s="10">
+        <v>37134</v>
+      </c>
     </row>
-    <row r="84" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B84" s="9">
         <v>14362</v>
@@ -77010,10 +77835,13 @@
       <c r="CM84" s="9">
         <v>35533</v>
       </c>
+      <c r="CN84" s="9">
+        <v>34781</v>
+      </c>
     </row>
-    <row r="85" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B85" s="10">
         <v>19045</v>
@@ -77285,10 +78113,13 @@
       <c r="CM85" s="10">
         <v>49227</v>
       </c>
+      <c r="CN85" s="10">
+        <v>47363</v>
+      </c>
     </row>
-    <row r="86" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B86" s="9">
         <v>10636</v>
@@ -77560,10 +78391,13 @@
       <c r="CM86" s="9">
         <v>28914</v>
       </c>
+      <c r="CN86" s="9">
+        <v>28238</v>
+      </c>
     </row>
-    <row r="87" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B87" s="10">
         <v>6154</v>
@@ -77835,10 +78669,13 @@
       <c r="CM87" s="10">
         <v>16654</v>
       </c>
+      <c r="CN87" s="10">
+        <v>15770</v>
+      </c>
     </row>
-    <row r="88" spans="1:91" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:92" s="1" customFormat="1" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B88" s="11">
         <v>52597</v>
@@ -78110,10 +78947,13 @@
       <c r="CM88" s="11">
         <v>134868</v>
       </c>
+      <c r="CN88" s="11">
+        <v>135675</v>
+      </c>
     </row>
-    <row r="89" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B89" s="10">
         <v>4597</v>
@@ -78385,10 +79225,13 @@
       <c r="CM89" s="10">
         <v>15069</v>
       </c>
+      <c r="CN89" s="10">
+        <v>15556</v>
+      </c>
     </row>
-    <row r="90" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B90" s="9">
         <v>7305</v>
@@ -78660,10 +79503,13 @@
       <c r="CM90" s="9">
         <v>18316</v>
       </c>
+      <c r="CN90" s="9">
+        <v>19224</v>
+      </c>
     </row>
-    <row r="91" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B91" s="10">
         <v>5159</v>
@@ -78935,10 +79781,13 @@
       <c r="CM91" s="10">
         <v>15336</v>
       </c>
+      <c r="CN91" s="10">
+        <v>14731</v>
+      </c>
     </row>
-    <row r="92" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B92" s="9">
         <v>2750</v>
@@ -79210,10 +80059,13 @@
       <c r="CM92" s="9">
         <v>6357</v>
       </c>
+      <c r="CN92" s="9">
+        <v>6437</v>
+      </c>
     </row>
-    <row r="93" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B93" s="10">
         <v>12124</v>
@@ -79485,10 +80337,13 @@
       <c r="CM93" s="10">
         <v>30155</v>
       </c>
+      <c r="CN93" s="10">
+        <v>30023</v>
+      </c>
     </row>
-    <row r="94" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B94" s="9">
         <v>9027</v>
@@ -79760,10 +80615,13 @@
       <c r="CM94" s="9">
         <v>21390</v>
       </c>
+      <c r="CN94" s="9">
+        <v>21570</v>
+      </c>
     </row>
-    <row r="95" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B95" s="10">
         <v>4665</v>
@@ -80035,10 +80893,13 @@
       <c r="CM95" s="10">
         <v>12033</v>
       </c>
+      <c r="CN95" s="10">
+        <v>11930</v>
+      </c>
     </row>
-    <row r="96" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B96" s="9">
         <v>1538</v>
@@ -80310,10 +81171,13 @@
       <c r="CM96" s="9">
         <v>3253</v>
       </c>
+      <c r="CN96" s="9">
+        <v>3316</v>
+      </c>
     </row>
-    <row r="97" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B97" s="10">
         <v>4152</v>
@@ -80585,10 +81449,13 @@
       <c r="CM97" s="10">
         <v>9704</v>
       </c>
+      <c r="CN97" s="10">
+        <v>9534</v>
+      </c>
     </row>
-    <row r="98" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B98" s="9">
         <v>826</v>
@@ -80860,10 +81727,13 @@
       <c r="CM98" s="9">
         <v>1949</v>
       </c>
+      <c r="CN98" s="9">
+        <v>2004</v>
+      </c>
     </row>
-    <row r="99" spans="1:91" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:92" s="1" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B99" s="10">
         <v>454</v>
@@ -81134,6 +82004,9 @@
       </c>
       <c r="CM99" s="10">
         <v>1308</v>
+      </c>
+      <c r="CN99" s="10">
+        <v>1349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>